<commit_message>
v4 Phase 3: fix package.py fieldnames crash on mixed NEW/REPEAT rows
</commit_message>
<xml_diff>
--- a/results/joey/LATAM/Week_of_2026-07-20/LATAM_Joey_Complete_2026-07-20.xlsx
+++ b/results/joey/LATAM/Week_of_2026-07-20/LATAM_Joey_Complete_2026-07-20.xlsx
@@ -426,10 +426,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z14"/>
+  <dimension ref="A1:Z18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
@@ -453,7 +453,7 @@
     <col width="18" customWidth="1" min="22" max="22"/>
     <col width="17" customWidth="1" min="23" max="23"/>
     <col width="31" customWidth="1" min="24" max="24"/>
-    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="31" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
@@ -976,22 +976,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>portfolio_board:qed-investors</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>firecrawl</t>
+          <t>caribou</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Firecrawl</t>
+          <t>Caribou</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Head of Growth Marketing</t>
+          <t>Senior Manager, Go-To-Market Operations &amp; Sales Tools</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>San Francisco, CA (Hybrid) OR Remote (Americas, UTC-3 to UTC-10)</t>
+          <t>Chicago, IL, Denver, CO, Phoenix, AZ, Remote, US</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -1056,29 +1056,21 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/firecrawl/252206c1-56a2-4598-abef-d2ed9e2295de</t>
+          <t>https://job-boards.greenhouse.io/caribou/jobs/7801514003</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2026-07-13T00:04:16.535+00:00</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>Ashby</t>
-        </is>
-      </c>
+          <t>2026-07-10T15:04:27Z</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>api-live</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
@@ -1087,12 +1079,12 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>jd_cache/14ad0946e1c31f94.txt</t>
+          <t>jd_cache/4bc951a8358c0c77.txt</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>portfolio_board:qed-investors</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
@@ -1109,27 +1101,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>gitlab</t>
+          <t>firecrawl</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Gitlab</t>
+          <t>Firecrawl</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Senior Program Manager, Enterprise Technology &amp; AI</t>
+          <t>Head of Growth Marketing</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>program</t>
+          <t>growth_commercial</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Remote, Bangalore</t>
+          <t>San Francisco, CA (Hybrid) OR Remote (Americas, UTC-3 to UTC-10)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1174,7 +1166,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1184,17 +1176,17 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gitlab/jobs/8584282002</t>
+          <t>https://jobs.ashbyhq.com/firecrawl/252206c1-56a2-4598-abef-d2ed9e2295de</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>2026-07-06T08:34:18-04:00</t>
+          <t>2026-07-13T00:04:16.535+00:00</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>Ashby</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1215,7 +1207,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>jd_cache/0516b4bb5d9aae63.txt</t>
+          <t>jd_cache/14ad0946e1c31f94.txt</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1247,17 +1239,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Vice President, Finance Strategy &amp; Operations</t>
+          <t>Senior Program Manager, Enterprise Technology &amp; AI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>strategic_ops</t>
+          <t>program</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Remote, US</t>
+          <t>Remote, Bangalore</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1312,12 +1304,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gitlab/jobs/8467198002</t>
+          <t>https://job-boards.greenhouse.io/gitlab/jobs/8584282002</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>2026-06-05T16:18:10-04:00</t>
+          <t>2026-07-06T08:34:18-04:00</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1343,7 +1335,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>jd_cache/b1fbef6c443cfc44.txt</t>
+          <t>jd_cache/0516b4bb5d9aae63.txt</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1365,27 +1357,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hightouch</t>
+          <t>gitlab</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hightouch</t>
+          <t>Gitlab</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Go-to-Market Engineer</t>
+          <t>Vice President, Finance Strategy &amp; Operations</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>growth_commercial</t>
+          <t>strategic_ops</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Remote, United States</t>
+          <t>Remote, US</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1430,7 +1422,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1440,12 +1432,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/hightouch/jobs/5823552004</t>
+          <t>https://job-boards.greenhouse.io/gitlab/jobs/8467198002</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>2026-06-16T17:07:05-04:00</t>
+          <t>2026-06-05T16:18:10-04:00</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1471,7 +1463,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>jd_cache/0e0db98a00b191dc.txt</t>
+          <t>jd_cache/b1fbef6c443cfc44.txt</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -2128,32 +2120,32 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>portfolio_board:a16z</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>upwork</t>
+          <t>stripe</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Upwork</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sr Director, Corporate Development</t>
+          <t>Strategic Programs Lead, New Markets</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>growth_commercial</t>
+          <t>strategic_ops</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Palo Alto, California, United States; Remote</t>
+          <t>US-Remote</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2208,29 +2200,21 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/upwork/jobs/7110133003</t>
+          <t>https://stripe.com/jobs/search?gh_jid=8070648</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>2026-05-11T14:20:37-04:00</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
+          <t>2026-07-16T21:33:48Z</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>api-live</t>
-        </is>
-      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
@@ -2239,15 +2223,495 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
+          <t>jd_cache/27c007c7f953372d.txt</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>portfolio_board:a16z</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>api</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>upwork</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Upwork</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Sr Director, Corporate Development</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>growth_commercial</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Palo Alto, California, United States; Remote</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>L?, D?, P?</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>needs_verification</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/upwork/jobs/7110133003</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>2026-05-11T14:20:37-04:00</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>api-live</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
           <t>jd_cache/4421f1e7876e2e3f.txt</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
+      <c r="Y15" t="inlineStr">
         <is>
           <t>api</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr">
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>portfolio_board:qed-investors</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>caliza</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>caliza</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Mexico - Director of Business Development</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>partnerships_bd</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Mexico City</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/caliza-financial-technologies/d3c4c930-0549-4dff-8b09-1fa9bee518a4</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>2026-05-08T05:45:51.939000Z</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>jd_cache/e68b8ab33da2203c.txt</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>portfolio_board:qed-investors</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>portfolio_board:a16z</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>talkiatry</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>talkiatry</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>General Manager/Director of Clinical Operations, Psychiatry</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>market_entry</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>United States, Remote</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>L?, D?, P?</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/talkiatry/f13dbc0c-63b4-4e75-bf24-91f0c87ce3e5?utm_source=jobs.a16z.com</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>2026-07-15T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>jd_cache/db072d64e2033f6d.txt</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>portfolio_board:a16z</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>portfolio_board:kaszek</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>wellhub</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>wellhub</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Partnerships Director – US National Partnerships</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>partnerships_bd</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>US (Remote)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>L?, D?, P?</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/gympass/jobs/8444113002</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>2026-03-05T23:49:33Z</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>jd_cache/246f403e48ce2b1d.txt</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>portfolio_board:kaszek</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
         <is>
           <t>REPEAT</t>
         </is>
@@ -2264,21 +2728,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:X9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="43" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="23" customWidth="1" min="15" max="15"/>
@@ -2287,7 +2751,7 @@
     <col width="27" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="15" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="45" customWidth="1" min="21" max="21"/>
     <col width="18" customWidth="1" min="22" max="22"/>
     <col width="17" customWidth="1" min="23" max="23"/>
     <col width="15" customWidth="1" min="24" max="24"/>
@@ -2528,6 +2992,748 @@
         </is>
       </c>
       <c r="X2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>portfolio_board:a16z</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>revolut</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Revolut</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Strategy &amp; Operations Manager</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>strategic_ops</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Australia - Remote, Australia</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>L?, D?, P?</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>fintech,financial-services</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>late-stage</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>https://www.revolut.com/en-US/careers/position/3c41a74a-d391-4cec-986b-066b43af038c/</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>2026-07-15T05:58:03Z</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>HTTP 403</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>http_error</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>portfolio_board:kaszek</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>arq</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ARQ (formerly DolarApp)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Head of Growth - Mexico</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>growth_commercial</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Mexico City, Mexico , Mexico, Mexico City</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>fintech</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>series-b</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/ARQ/7c7d8951-7b71-403d-a21a-efde6d306e8d</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2026-04-22T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>stale</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Ashby API: posted 89d ago (2026-04-22)</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>portfolio_board:kaszek</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>arq</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ARQ (formerly DolarApp)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Head of Growth - Colombia</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>growth_commercial</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Bogota, Colombia, Colombia, Bogota</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>fintech</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>series-b</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/ARQ/bb1a6458-6003-4082-98a0-8ec61d3049b4</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2026-04-22T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>stale</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Ashby API: posted 89d ago (2026-04-22)</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>portfolio_board:kaszek</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>pomelo</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Pomelo</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Country Manager COL</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>market_entry</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Bogotá, Bogotá, Colombia</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>https://pomelo.la/en/work-with-us?gh_jid=5833410004</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>2026-04-22T18:08:30Z</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>no job ID in URL path</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>portfolio_board:a16z</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>thatch</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>thatch</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Strategy and Operations Manager</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>strategic_ops</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Austin, Texas, United States, Remote (US)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>L, D, P?</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>https://thatch.com/jobs/5358702008?gh_jid=5358702008</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>2026-07-16T21:23:14Z</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>HTTP 404</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>portfolio_board:a16z</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>anduril-industries</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>anduril-industries</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Senior Program Manager, People Operations</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>program</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>L?, D?, P?</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/andurilindustries/jobs/5188733007?gh_jid=5188733007</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:35:21Z</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>cross-domain redirect: job-boards.greenhouse.io</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>portfolio_board:a16z</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>thatch</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>thatch</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Channel Partnerships Manager</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>partnerships_bd</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>L, D, P?</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>https://thatch.com/jobs/5358793008?gh_jid=5358793008</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:16:39Z</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>HTTP 404</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2578,7 +3784,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -2588,7 +3794,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -2598,7 +3804,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -2608,7 +3814,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -2618,7 +3824,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -2638,7 +3844,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -2658,7 +3864,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Run 2026-07-22 weekly LATAM search; update README with v4 rebuild milestone
Full run.py pipeline: 115 companies checked, 3225 jobs scanned, 19
candidates through health check, 18/19 JDs fetched (95%), 17 scored.
claude-p backend hit repeated 120s subprocess timeouts on 3 of 4
scoring batches this run; rescored via the API backend (tool-forced
structured output) for a clean 17/17. Top score 47 (Caliza, Mexico
City) — below the 60+ cutoff, an honest result given the corpus isn't
LATAM-enriched yet (Phase 3 sourcing work covers recall, not scoring
bias). Master list grew by 2 new rows.

README: added a Week 13 entry documenting the v4 rebuild (Phase 0-3)
completed this month, and updated the R&D track description.
</commit_message>
<xml_diff>
--- a/results/joey/LATAM/Week_of_2026-07-20/LATAM_Joey_Complete_2026-07-20.xlsx
+++ b/results/joey/LATAM/Week_of_2026-07-20/LATAM_Joey_Complete_2026-07-20.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +43,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F2A44"/>
         <bgColor rgb="001F2A44"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F2E1"/>
+        <bgColor rgb="00E3F2E1"/>
       </patternFill>
     </fill>
   </fills>
@@ -58,9 +64,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z18"/>
+  <dimension ref="A1:AA18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -455,6 +462,7 @@
     <col width="31" customWidth="1" min="24" max="24"/>
     <col width="31" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="17" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -588,6 +596,11 @@
           <t>status</t>
         </is>
       </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>first_seen_week</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -716,6 +729,7 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -844,6 +858,7 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -972,6 +987,7 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1092,6 +1108,7 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1220,6 +1237,7 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1348,6 +1366,7 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1476,6 +1495,7 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1485,17 +1505,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>includedhealth</t>
+          <t>hightouch</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Includedhealth</t>
+          <t>Hightouch</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Go-To-Market Enablement Manager</t>
+          <t>Go-to-Market Engineer</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1505,7 +1525,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Remote, United States</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1560,17 +1580,17 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/includedhealth/e5475693-8b26-4166-ad01-db9bcbbf2f96</t>
+          <t>https://job-boards.greenhouse.io/hightouch/jobs/5823552004</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>2026-06-26T15:26:50.581000</t>
+          <t>2026-06-16T17:07:05-04:00</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Lever</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1591,7 +1611,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>jd_cache/9f6400b899262c75.txt</t>
+          <t>jd_cache/0e0db98a00b191dc.txt</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -1604,6 +1624,7 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1613,27 +1634,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>nift</t>
+          <t>includedhealth</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Nift</t>
+          <t>Includedhealth</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">General Manager, EMEA / UK </t>
+          <t>Go-To-Market Enablement Manager</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>market_entry</t>
+          <t>growth_commercial</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Remote, UK</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1688,17 +1709,17 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/nift/jobs/4917411007</t>
+          <t>https://jobs.lever.co/includedhealth/e5475693-8b26-4166-ad01-db9bcbbf2f96</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>2026-01-13T16:05:47-05:00</t>
+          <t>2026-06-26T15:26:50.581000</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>Lever</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1719,7 +1740,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>jd_cache/61bf1cb46e9a777e.txt</t>
+          <t>jd_cache/9f6400b899262c75.txt</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -1732,6 +1753,7 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1741,27 +1763,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>pivotal-health</t>
+          <t>nift</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pivotal Health</t>
+          <t>Nift</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Client Strategy &amp; Operations Manager</t>
+          <t xml:space="preserve">General Manager, EMEA / UK </t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>strategic_ops</t>
+          <t>market_entry</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Remote - NY</t>
+          <t>Remote, UK</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1806,7 +1828,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1816,17 +1838,17 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/pivotal-health/ce4e43d1-7add-408b-ae2d-c1205509527d</t>
+          <t>https://job-boards.greenhouse.io/nift/jobs/4917411007</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>2026-05-20T22:25:49.748+00:00</t>
+          <t>2026-01-13T16:05:47-05:00</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Ashby</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1847,7 +1869,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>jd_cache/00f0fa111ce5ea70.txt</t>
+          <t>jd_cache/61bf1cb46e9a777e.txt</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -1860,6 +1882,7 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1869,27 +1892,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>remotecom</t>
+          <t>pivotal-health</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Remotecom</t>
+          <t>Pivotal Health</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Global Payroll Implementation Country Lead - Germany</t>
+          <t>Client Strategy &amp; Operations Manager</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>market_entry</t>
+          <t>strategic_ops</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Remote - DACH</t>
+          <t>Remote - NY</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1914,7 +1937,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>none</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1934,7 +1957,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1944,17 +1967,17 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/remotecom/jobs/7735395003</t>
+          <t>https://jobs.ashbyhq.com/pivotal-health/ce4e43d1-7add-408b-ae2d-c1205509527d</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>2026-05-20T12:43:07-04:00</t>
+          <t>2026-05-20T22:25:49.748+00:00</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>Ashby</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1975,7 +1998,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>jd_cache/64301db3564e8a84.txt</t>
+          <t>jd_cache/00f0fa111ce5ea70.txt</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -1988,154 +2011,160 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>api</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>rula</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Rula</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Strategy &amp; Operations Manager  (Remote)</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>strategic_ops</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Remote - United States</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>L?, D?, P?</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>remotecom</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Remotecom</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Global Payroll Implementation Country Lead - Germany</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>market_entry</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Remote - EMEA</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
         <is>
           <t>needs_verification</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/rula/3013fcdb-0e71-42f2-b3f1-7e8e3b3a2c44</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>2026-06-18T19:42:02.894+00:00</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>Ashby</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/remotecom/jobs/7741670003</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20T12:43:21-04:00</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="U13" s="2" t="inlineStr">
         <is>
           <t>api-live</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr">
+      <c r="V13" s="2" t="inlineStr"/>
+      <c r="W13" s="2" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>jd_cache/8b31a0d5dbd4b5fb.txt</t>
-        </is>
-      </c>
-      <c r="Y13" t="inlineStr">
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>jd_cache/6942018b9b8aad47.txt</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
         <is>
           <t>api</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>REPEAT</t>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>portfolio_board:a16z</t>
+          <t>api</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>stripe</t>
+          <t>rula</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>Rula</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Strategic Programs Lead, New Markets</t>
+          <t>Strategy &amp; Operations Manager  (Remote)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -2145,7 +2174,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>US-Remote</t>
+          <t>Remote - United States</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2200,21 +2229,29 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>https://stripe.com/jobs/search?gh_jid=8070648</t>
+          <t>https://jobs.ashbyhq.com/rula/3013fcdb-0e71-42f2-b3f1-7e8e3b3a2c44</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>2026-07-16T21:33:48Z</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr"/>
+          <t>2026-06-18T19:42:02.894+00:00</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Ashby</t>
+        </is>
+      </c>
       <c r="T14" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>api-live</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
@@ -2223,12 +2260,12 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>jd_cache/27c007c7f953372d.txt</t>
+          <t>jd_cache/8b31a0d5dbd4b5fb.txt</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>portfolio_board:a16z</t>
+          <t>api</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -2236,184 +2273,182 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>api</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>upwork</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Upwork</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Sr Director, Corporate Development</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>growth_commercial</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Palo Alto, California, United States; Remote</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_board:a16z</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>stripe</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Strategy and Operations Lead, Deal Pricing</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>strategic_ops</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>US-Remote</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>L?, D?, P?</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="P15" s="2" t="inlineStr">
         <is>
           <t>needs_verification</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/upwork/jobs/7110133003</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>2026-05-11T14:20:37-04:00</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>https://stripe.com/jobs/search?gh_jid=8044391</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20T22:43:18Z</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>api-live</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr">
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="2" t="inlineStr"/>
+      <c r="W15" s="2" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>jd_cache/4421f1e7876e2e3f.txt</t>
-        </is>
-      </c>
-      <c r="Y15" t="inlineStr">
-        <is>
-          <t>api</t>
-        </is>
-      </c>
-      <c r="Z15" t="inlineStr">
-        <is>
-          <t>REPEAT</t>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>jd_cache/25de98b90637aedf.txt</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_board:a16z</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>portfolio_board:qed-investors</t>
+          <t>api</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>caliza</t>
+          <t>upwork</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>caliza</t>
+          <t>Upwork</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Mexico - Director of Business Development</t>
+          <t>Sr Director, Corporate Development</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>partnerships_bd</t>
+          <t>growth_commercial</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Palo Alto, California, United States; Remote</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>L?, D?, P?</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>unclear</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>unclear</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>unclear</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2421,7 +2456,11 @@
           <t>none</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
           <t>unknown</t>
@@ -2439,26 +2478,34 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>needs_verification</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/caliza-financial-technologies/d3c4c930-0549-4dff-8b09-1fa9bee518a4</t>
+          <t>https://job-boards.greenhouse.io/upwork/jobs/7110133003</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>2026-05-08T05:45:51.939000Z</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr"/>
+          <t>2026-05-11T14:20:37-04:00</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
       <c r="T16" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>api-live</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
@@ -2467,12 +2514,12 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>jd_cache/e68b8ab33da2203c.txt</t>
+          <t>jd_cache/4421f1e7876e2e3f.txt</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>portfolio_board:qed-investors</t>
+          <t>api</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
@@ -2480,56 +2527,57 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>portfolio_board:a16z</t>
+          <t>portfolio_board:qed-investors</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>talkiatry</t>
+          <t>caliza</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>talkiatry</t>
+          <t>caliza</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>General Manager/Director of Clinical Operations, Psychiatry</t>
+          <t>Mexico - Director of Business Development</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>market_entry</t>
+          <t>partnerships_bd</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>United States, Remote</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>L?, D?, P?</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>true</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>false</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>false</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2560,12 +2608,12 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/talkiatry/f13dbc0c-63b4-4e75-bf24-91f0c87ce3e5?utm_source=jobs.a16z.com</t>
+          <t>https://jobs.lever.co/caliza-financial-technologies/d3c4c930-0549-4dff-8b09-1fa9bee518a4</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>2026-07-15T00:00:00Z</t>
+          <t>2026-05-08T05:45:51.939000Z</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
@@ -2575,11 +2623,7 @@
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
+      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr">
         <is>
           <t>success</t>
@@ -2587,12 +2631,12 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>jd_cache/db072d64e2033f6d.txt</t>
+          <t>jd_cache/e68b8ab33da2203c.txt</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>portfolio_board:a16z</t>
+          <t>portfolio_board:qed-investors</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
@@ -2600,36 +2644,37 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>portfolio_board:kaszek</t>
+          <t>portfolio_board:a16z</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>wellhub</t>
+          <t>talkiatry</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>wellhub</t>
+          <t>talkiatry</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Partnerships Director – US National Partnerships</t>
+          <t>General Manager/Director of Clinical Operations, Psychiatry</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>partnerships_bd</t>
+          <t>market_entry</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>US (Remote)</t>
+          <t>United States, Remote</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2680,12 +2725,12 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gympass/jobs/8444113002</t>
+          <t>https://jobs.ashbyhq.com/talkiatry/f13dbc0c-63b4-4e75-bf24-91f0c87ce3e5?utm_source=jobs.a16z.com</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>2026-03-05T23:49:33Z</t>
+          <t>2026-07-15T00:00:00Z</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
@@ -2695,7 +2740,11 @@
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="W18" t="inlineStr">
         <is>
           <t>success</t>
@@ -2703,12 +2752,12 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>jd_cache/246f403e48ce2b1d.txt</t>
+          <t>jd_cache/db072d64e2033f6d.txt</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>portfolio_board:kaszek</t>
+          <t>portfolio_board:a16z</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
@@ -2716,6 +2765,7 @@
           <t>REPEAT</t>
         </is>
       </c>
+      <c r="AA18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2728,7 +2778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X9"/>
+  <dimension ref="A1:X6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2742,7 +2792,7 @@
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="23" customWidth="1" min="15" max="15"/>
@@ -2967,7 +3017,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2026-06-17T22:01:46-04:00</t>
+          <t>2026-07-21T17:18:10-04:00</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -2996,52 +3046,52 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>portfolio_board:a16z</t>
+          <t>portfolio_board:kaszek</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>revolut</t>
+          <t>arq</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Revolut</t>
+          <t>ARQ (formerly DolarApp)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Manager</t>
+          <t>Head of Growth - Mexico</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>strategic_ops</t>
+          <t>growth_commercial</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Australia - Remote, Australia</t>
+          <t>Mexico City, Mexico , Mexico, Mexico City</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>L?, D?, P?</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>true</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>false</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>false</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -3051,56 +3101,56 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>fintech,financial-services</t>
+          <t>fintech</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>late-stage</t>
+          <t>series-b</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>https://www.revolut.com/en-US/careers/position/3c41a74a-d391-4cec-986b-066b43af038c/</t>
+          <t>https://jobs.ashbyhq.com/ARQ/7c7d8951-7b71-403d-a21a-efde6d306e8d</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2026-07-15T05:58:03Z</t>
+          <t>2026-04-22T00:00:00Z</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>stale</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>HTTP 403</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>http_error</t>
-        </is>
-      </c>
+          <t>Ashby API: posted 91d ago (2026-04-22)</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -3111,27 +3161,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>arq</t>
+          <t>pomelo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ARQ (formerly DolarApp)</t>
+          <t>Pomelo</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Head of Growth - Mexico</t>
+          <t>Country Manager COL</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>growth_commercial</t>
+          <t>market_entry</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico , Mexico, Mexico City</t>
+          <t>Bogotá, Bogotá, Colombia</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -3156,97 +3206,93 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>fintech</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>series-b</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/ARQ/7c7d8951-7b71-403d-a21a-efde6d306e8d</t>
+          <t>https://pomelo.la/en/work-with-us?gh_jid=5833410004</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>2026-04-22T00:00:00Z</t>
+          <t>2026-04-22T18:08:30Z</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>stale</t>
+          <t>generic</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Ashby API: posted 89d ago (2026-04-22)</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
-      </c>
+          <t>no job ID in URL path</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>portfolio_board:kaszek</t>
+          <t>portfolio_board:a16z</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>arq</t>
+          <t>thatch</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ARQ (formerly DolarApp)</t>
+          <t>thatch</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Head of Growth - Colombia</t>
+          <t>Strategy and Operations Manager</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>growth_commercial</t>
+          <t>strategic_ops</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Bogota, Colombia, Colombia, Bogota</t>
+          <t>Austin, Texas, United States, Remote (US)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>L, D, P?</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -3256,12 +3302,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>unclear</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -3269,121 +3315,109 @@
           <t>none</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>fintech</t>
-        </is>
-      </c>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>series-b</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/ARQ/bb1a6458-6003-4082-98a0-8ec61d3049b4</t>
+          <t>https://thatch.com/jobs/5358702008?gh_jid=5358702008</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2026-04-22T00:00:00Z</t>
+          <t>2026-07-16T21:23:14Z</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>stale</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Ashby API: posted 89d ago (2026-04-22)</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
-      </c>
+          <t>HTTP 404</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>portfolio_board:kaszek</t>
+          <t>portfolio_board:a16z</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>pomelo</t>
+          <t>anduril-industries</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pomelo</t>
+          <t>anduril-industries</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Country Manager COL</t>
+          <t>Senior Program Manager, People Operations</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>market_entry</t>
+          <t>program</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Bogotá, Bogotá, Colombia</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>L?, D?, P?</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>unclear</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>unclear</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>unclear</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>direct</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
           <t>unknown</t>
@@ -3396,7 +3430,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -3406,334 +3440,28 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>https://pomelo.la/en/work-with-us?gh_jid=5833410004</t>
+          <t>https://boards.greenhouse.io/andurilindustries/jobs/5188733007?gh_jid=5188733007</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>2026-04-22T18:08:30Z</t>
+          <t>2026-07-16T12:35:21Z</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>generic</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>no job ID in URL path</t>
+          <t>cross-domain redirect: job-boards.greenhouse.io</t>
         </is>
       </c>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>portfolio_board:a16z</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>thatch</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>thatch</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Strategy and Operations Manager</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>strategic_ops</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Austin, Texas, United States, Remote (US)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>L, D, P?</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>https://thatch.com/jobs/5358702008?gh_jid=5358702008</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>2026-07-16T21:23:14Z</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>closed</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>HTTP 404</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>portfolio_board:a16z</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>anduril-industries</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>anduril-industries</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Senior Program Manager, People Operations</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>program</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>L?, D?, P?</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/andurilindustries/jobs/5188733007?gh_jid=5188733007</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>2026-07-16T12:35:21Z</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>closed</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>cross-domain redirect: job-boards.greenhouse.io</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>portfolio_board:a16z</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>thatch</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>thatch</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Channel Partnerships Manager</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>partnerships_bd</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Remote (US)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>L, D, P?</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>https://thatch.com/jobs/5358793008?gh_jid=5358793008</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>2026-07-16T12:16:39Z</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>closed</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>HTTP 404</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3784,7 +3512,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -3804,7 +3532,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -3814,7 +3542,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -3834,7 +3562,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -3844,7 +3572,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -3854,7 +3582,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -3864,7 +3592,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>